<commit_message>
Add Ukrainian TouchRetouch deliverables + fix xlsx note bug
Fix #ERROR! in the EN model (note cells starting with '=' were parsed
as formulas). Add Ukrainian versions of all three files (xlsx 4 sheets,
12-slide deck, doc) restyled with a warmer, less-templated look:
serif headings, eyebrow+rule instead of solid bars, first-person voice.

https://claude.ai/code/session_01NksSqrSqDgtmZbhunqjgZD
</commit_message>
<xml_diff>
--- a/outputs/touchretouch-testtask/TouchRetouch_ASA_ROAS_Model.xlsx
+++ b/outputs/touchretouch-testtask/TouchRetouch_ASA_ROAS_Model.xlsx
@@ -789,9 +789,10 @@
         <f>$B$6*$B$7</f>
         <v/>
       </c>
-      <c r="D13" s="9">
-        <f> trial% × paid%</f>
-        <v/>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>trial% × paid%</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -804,9 +805,10 @@
         <f>$B$13*$B$8</f>
         <v/>
       </c>
-      <c r="D14" s="9">
-        <f> payers/install × ARPPU</f>
-        <v/>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>payers/install × ARPPU</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -819,9 +821,10 @@
         <f>$B$14</f>
         <v/>
       </c>
-      <c r="D15" s="9">
-        <f> revenue per install</f>
-        <v/>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>revenue per install</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -834,9 +837,10 @@
         <f>$B$14/$B$10</f>
         <v/>
       </c>
-      <c r="D16" s="9">
-        <f> rev/install ÷ min ROAS</f>
-        <v/>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>rev/install ÷ min ROAS</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -1388,7 +1392,7 @@
         </is>
       </c>
       <c r="B5" s="27" t="n">
-        <v>0.078</v>
+        <v>0.42</v>
       </c>
       <c r="C5" s="27">
         <f>B5*1.1</f>

</xml_diff>